<commit_message>
fix: fix en bdd de jugadores
</commit_message>
<xml_diff>
--- a/backend/src/db/Jugadores_Historico.xlsx
+++ b/backend/src/db/Jugadores_Historico.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carreño\Documents\Nico\Git\Brumario\backend\src\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Documents\GitHub\Brumario\backend\src\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEFEDE2F-B9AE-421F-B996-882D7E57D088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7050"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
   <si>
     <t>Nombre</t>
   </si>
@@ -516,12 +517,15 @@
   </si>
   <si>
     <t>Yafar, Yamil</t>
+  </si>
+  <si>
+    <t>2Giménez, Ariel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -614,7 +618,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -891,834 +895,834 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:B166"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="30.28515625" customWidth="1"/>
+    <col min="2" max="2" width="30.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B21" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B22" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B23" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B24" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B25" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B26" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B27" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B28" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B29" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B30" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B31" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B32" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B33" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B34" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B35" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B36" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B37" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B38" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B39" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B40" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B41" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B42" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B43" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B44" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B45" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B46" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B47" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B48" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B49" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B51" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B52" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B53" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B54" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B55" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B56" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B57" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B58" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B59" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B60" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B61" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B62" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B63" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B64" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B65" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B66" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B67" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B68" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B69" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B70" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B71" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B72" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B73" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B74" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B75" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B76" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B77" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B78" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B79" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B80" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B81" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B82" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B83" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B84" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B85" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B86" s="1" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B87" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B88" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B89" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B90" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B91" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B92" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B93" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B94" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B95" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B96" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B97" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B98" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B99" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B100" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B101" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B102" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B103" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B104" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B105" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B106" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B107" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B108" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B109" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B110" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B111" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B112" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B113" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B114" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B115" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B116" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B117" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B118" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B119" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B120" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B121" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B122" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B123" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B124" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B125" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B126" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B127" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B128" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B129" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B130" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B131" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B132" s="1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B133" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B134" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B135" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B136" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B137" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B138" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B139" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B140" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B141" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B142" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B143" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B144" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B145" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B146" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B147" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B148" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B149" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B150" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B151" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B152" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B153" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B154" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B155" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B156" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B157" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B158" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B159" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B160" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B161" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B162" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B163" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B164" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B165" s="1" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B166" s="3" t="s">
         <v>163</v>
       </c>

</xml_diff>

<commit_message>
feat: hitos jugador (completado)
agrego debut y debut oficial
</commit_message>
<xml_diff>
--- a/backend/src/db/Jugadores_Historico.xlsx
+++ b/backend/src/db/Jugadores_Historico.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Documents\GitHub\Brumario\backend\src\db\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Documents\Nico\brumario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEFEDE2F-B9AE-421F-B996-882D7E57D088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54221394-C181-4ABF-A221-472230963769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="168">
   <si>
     <t>Nombre</t>
   </si>
@@ -517,6 +517,15 @@
   </si>
   <si>
     <t>Yafar, Yamil</t>
+  </si>
+  <si>
+    <t>Debut</t>
+  </si>
+  <si>
+    <t>Debut Oficial</t>
+  </si>
+  <si>
+    <t>Dorsal</t>
   </si>
   <si>
     <t>2Giménez, Ariel</t>
@@ -526,7 +535,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -545,15 +558,46 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FF00FF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -604,7 +648,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -613,6 +657,54 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -896,838 +988,1625 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:B166"/>
+  <dimension ref="B2:E166"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="30.26953125" customWidth="1"/>
+    <col min="3" max="3" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C11" s="5">
+        <v>45472</v>
+      </c>
+      <c r="D11" s="5">
+        <v>45472</v>
+      </c>
+      <c r="E11" s="4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C13" s="5">
+        <v>45361</v>
+      </c>
+      <c r="D13" s="5">
+        <v>45396</v>
+      </c>
+      <c r="E13" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C14" s="5">
+        <v>45164</v>
+      </c>
+      <c r="D14" s="5">
+        <v>45200</v>
+      </c>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C17" s="6">
+        <v>44422</v>
+      </c>
+      <c r="D17" s="6">
+        <v>44436</v>
+      </c>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C18" s="5">
+        <v>44793</v>
+      </c>
+      <c r="D18" s="5">
+        <v>44807</v>
+      </c>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C19" s="7">
+        <v>45220</v>
+      </c>
+      <c r="D19" s="7">
+        <v>45220</v>
+      </c>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C23" s="8">
+        <v>45346</v>
+      </c>
+      <c r="D23" s="8">
+        <v>45423</v>
+      </c>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C26" s="9">
+        <v>44739</v>
+      </c>
+      <c r="D26" s="9">
+        <v>44746</v>
+      </c>
+      <c r="E26" s="10">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C27" s="8">
+        <v>45164</v>
+      </c>
+      <c r="D27" s="11">
+        <v>45220</v>
+      </c>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B30" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C31" s="4"/>
+      <c r="D31" s="12">
+        <v>42161</v>
+      </c>
+      <c r="E31" s="13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B33" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C34" s="8">
+        <v>44758</v>
+      </c>
+      <c r="D34" s="8">
+        <v>44758</v>
+      </c>
+      <c r="E34" s="14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B37" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B38" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B39" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B40" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B41" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B42" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B43" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B44" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C44" s="8">
+        <v>45395</v>
+      </c>
+      <c r="D44" s="8">
+        <v>45423</v>
+      </c>
+      <c r="E44" s="14">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B45" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B46" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C46" s="12">
+        <v>43652</v>
+      </c>
+      <c r="D46" s="12">
+        <v>43722</v>
+      </c>
+      <c r="E46" s="13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B47" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B48" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C48" s="15">
+        <v>42294</v>
+      </c>
+      <c r="D48" s="12">
+        <v>42294</v>
+      </c>
+      <c r="E48" s="13">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B49" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B50" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B51" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C51" s="8">
+        <v>45395</v>
+      </c>
+      <c r="D51" s="8">
+        <v>45423</v>
+      </c>
+      <c r="E51" s="14">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B52" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C52" s="4"/>
+      <c r="D52" s="12">
+        <v>42161</v>
+      </c>
+      <c r="E52" s="13">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B53" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C53" s="9">
+        <v>44739</v>
+      </c>
+      <c r="D53" s="9">
+        <v>44746</v>
+      </c>
+      <c r="E53" s="10">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B54" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C54" s="8">
+        <v>43708</v>
+      </c>
+      <c r="D54" s="8">
+        <v>44716</v>
+      </c>
+      <c r="E54" s="13">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B55" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C55" s="8">
+        <v>44961</v>
+      </c>
+      <c r="D55" s="8">
+        <v>45038</v>
+      </c>
+      <c r="E55" s="13">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B56" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C56" s="8">
+        <v>45346</v>
+      </c>
+      <c r="D56" s="8">
+        <v>45423</v>
+      </c>
+      <c r="E56" s="14">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B57" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C57" s="8">
+        <v>45374</v>
+      </c>
+      <c r="D57" s="8">
+        <v>45423</v>
+      </c>
+      <c r="E57" s="4"/>
+    </row>
+    <row r="58" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B58" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B59" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C59" s="9">
+        <v>44226</v>
+      </c>
+      <c r="D59" s="9">
+        <v>44436</v>
+      </c>
+      <c r="E59" s="10">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B60" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+    </row>
+    <row r="61" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B61" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C61" s="4"/>
+      <c r="D61" s="12">
+        <v>42161</v>
+      </c>
+      <c r="E61" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B62" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+    </row>
+    <row r="63" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B63" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+    </row>
+    <row r="64" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B64" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B65" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B66" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C66" s="11">
+        <v>45255</v>
+      </c>
+      <c r="D66" s="11">
+        <v>45255</v>
+      </c>
+      <c r="E66" s="14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B67" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+    </row>
+    <row r="68" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B68" s="1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="4"/>
+    </row>
+    <row r="69" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B69" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C69" s="4"/>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+    </row>
+    <row r="70" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B70" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C70" s="12">
+        <v>43890</v>
+      </c>
+      <c r="D70" s="12">
+        <v>44436</v>
+      </c>
+      <c r="E70" s="13">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="71" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B71" s="1" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C71" s="8">
+        <v>45361</v>
+      </c>
+      <c r="D71" s="8">
+        <v>45403</v>
+      </c>
+      <c r="E71" s="4"/>
+    </row>
+    <row r="72" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B72" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C72" s="8">
+        <v>45417</v>
+      </c>
+      <c r="D72" s="8">
+        <v>45417</v>
+      </c>
+      <c r="E72" s="4"/>
+    </row>
+    <row r="73" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B73" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+    </row>
+    <row r="74" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B74" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="4"/>
+    </row>
+    <row r="75" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B75" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B76" s="1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="76" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B76" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="C76" s="4"/>
+      <c r="D76" s="4"/>
+      <c r="E76" s="4"/>
+    </row>
+    <row r="77" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B77" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+    </row>
+    <row r="78" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B78" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C78" s="4"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="4"/>
+    </row>
+    <row r="79" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B79" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+    </row>
+    <row r="80" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B80" s="1" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C80" s="11">
+        <v>45255</v>
+      </c>
+      <c r="D80" s="11">
+        <v>45255</v>
+      </c>
+      <c r="E80" s="14">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="81" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B81" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C81" s="12">
+        <v>41832</v>
+      </c>
+      <c r="D81" s="12">
+        <v>41832</v>
+      </c>
+      <c r="E81" s="13">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="82" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B82" s="1" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C82" s="4"/>
+      <c r="D82" s="4"/>
+      <c r="E82" s="4"/>
+    </row>
+    <row r="83" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B83" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+    </row>
+    <row r="84" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B84" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C84" s="4"/>
+      <c r="D84" s="4"/>
+      <c r="E84" s="4"/>
+    </row>
+    <row r="85" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B85" s="1" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C85" s="4"/>
+      <c r="D85" s="4"/>
+      <c r="E85" s="4"/>
+    </row>
+    <row r="86" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B86" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C86" s="4"/>
+      <c r="D86" s="4"/>
+      <c r="E86" s="4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B87" s="1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C87" s="4"/>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
+    </row>
+    <row r="88" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B88" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C88" s="4"/>
+      <c r="D88" s="4"/>
+      <c r="E88" s="4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="89" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B89" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C89" s="4"/>
+      <c r="D89" s="4"/>
+      <c r="E89" s="4"/>
+    </row>
+    <row r="90" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B90" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C90" s="4"/>
+      <c r="D90" s="4"/>
+      <c r="E90" s="4"/>
+    </row>
+    <row r="91" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B91" s="1" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C91" s="16">
+        <v>44723</v>
+      </c>
+      <c r="D91" s="16">
+        <v>44723</v>
+      </c>
+      <c r="E91" s="4"/>
+    </row>
+    <row r="92" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B92" s="1" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C92" s="4"/>
+      <c r="D92" s="4"/>
+      <c r="E92" s="4"/>
+    </row>
+    <row r="93" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B93" s="1" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C93" s="4"/>
+      <c r="D93" s="4"/>
+      <c r="E93" s="4"/>
+    </row>
+    <row r="94" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B94" s="1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C94" s="4"/>
+      <c r="D94" s="4"/>
+      <c r="E94" s="4"/>
+    </row>
+    <row r="95" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B95" s="1" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+    </row>
+    <row r="96" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B96" s="1" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C96" s="4"/>
+      <c r="D96" s="4"/>
+      <c r="E96" s="4"/>
+    </row>
+    <row r="97" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B97" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C97" s="4"/>
+      <c r="D97" s="4"/>
+      <c r="E97" s="4"/>
+    </row>
+    <row r="98" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B98" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C98" s="4"/>
+      <c r="D98" s="4"/>
+      <c r="E98" s="4"/>
+    </row>
+    <row r="99" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B99" s="1" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+    </row>
+    <row r="100" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B100" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C100" s="4"/>
+      <c r="D100" s="4"/>
+      <c r="E100" s="4"/>
+    </row>
+    <row r="101" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B101" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C101" s="4"/>
+      <c r="D101" s="4"/>
+      <c r="E101" s="4"/>
+    </row>
+    <row r="102" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B102" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C102" s="4"/>
+      <c r="D102" s="4"/>
+      <c r="E102" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B103" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C103" s="4"/>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+    </row>
+    <row r="104" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B104" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C104" s="4"/>
+      <c r="D104" s="4"/>
+      <c r="E104" s="4"/>
+    </row>
+    <row r="105" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B105" s="1" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C105" s="16">
+        <v>44961</v>
+      </c>
+      <c r="D105" s="16">
+        <v>45038</v>
+      </c>
+      <c r="E105" s="4"/>
+    </row>
+    <row r="106" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B106" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C106" s="8">
+        <v>45403</v>
+      </c>
+      <c r="D106" s="8">
+        <v>45403</v>
+      </c>
+      <c r="E106" s="14">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="107" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B107" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C107" s="8">
+        <v>45346</v>
+      </c>
+      <c r="D107" s="8">
+        <v>45423</v>
+      </c>
+      <c r="E107" s="14">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="108" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B108" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C108" s="4"/>
+      <c r="D108" s="4"/>
+      <c r="E108" s="4"/>
+    </row>
+    <row r="109" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B109" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C109" s="8">
+        <v>44961</v>
+      </c>
+      <c r="D109" s="8">
+        <v>45080</v>
+      </c>
+      <c r="E109" s="14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B110" s="1" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C110" s="4"/>
+      <c r="D110" s="4"/>
+      <c r="E110" s="4"/>
+    </row>
+    <row r="111" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B111" s="1" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C111" s="4"/>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+    </row>
+    <row r="112" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B112" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C112" s="4"/>
+      <c r="D112" s="4"/>
+      <c r="E112" s="4"/>
+    </row>
+    <row r="113" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B113" s="1" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C113" s="4"/>
+      <c r="D113" s="4"/>
+      <c r="E113" s="4"/>
+    </row>
+    <row r="114" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B114" s="1" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C114" s="4"/>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4"/>
+    </row>
+    <row r="115" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B115" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C115" s="8">
+        <v>45417</v>
+      </c>
+      <c r="D115" s="8">
+        <v>45417</v>
+      </c>
+      <c r="E115" s="14">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="116" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B116" s="1" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C116" s="4"/>
+      <c r="D116" s="4"/>
+      <c r="E116" s="4"/>
+    </row>
+    <row r="117" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B117" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C117" s="4"/>
+      <c r="D117" s="4"/>
+      <c r="E117" s="4"/>
+    </row>
+    <row r="118" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B118" s="1" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C118" s="8">
+        <v>45556</v>
+      </c>
+      <c r="D118" s="8">
+        <v>45556</v>
+      </c>
+      <c r="E118" s="4"/>
+    </row>
+    <row r="119" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B119" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C119" s="8">
+        <v>45273</v>
+      </c>
+      <c r="D119" s="8">
+        <v>45273</v>
+      </c>
+      <c r="E119" s="4"/>
+    </row>
+    <row r="120" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B120" s="1" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C120" s="4"/>
+      <c r="D120" s="4"/>
+      <c r="E120" s="4"/>
+    </row>
+    <row r="121" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B121" s="1" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C121" s="4"/>
+      <c r="D121" s="4"/>
+      <c r="E121" s="4"/>
+    </row>
+    <row r="122" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B122" s="1" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C122" s="4"/>
+      <c r="D122" s="4"/>
+      <c r="E122" s="4"/>
+    </row>
+    <row r="123" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B123" s="1" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C123" s="4"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+    </row>
+    <row r="124" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B124" s="1" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C124" s="4"/>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
+    </row>
+    <row r="125" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B125" s="1" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C125" s="17">
+        <v>44247</v>
+      </c>
+      <c r="D125" s="17">
+        <v>44436</v>
+      </c>
+      <c r="E125" s="13">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="126" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B126" s="1" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C126" s="4"/>
+      <c r="D126" s="4"/>
+      <c r="E126" s="4"/>
+    </row>
+    <row r="127" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B127" s="1" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C127" s="4"/>
+      <c r="D127" s="4"/>
+      <c r="E127" s="4"/>
+    </row>
+    <row r="128" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B128" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C128" s="4"/>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+    </row>
+    <row r="129" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B129" s="1" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C129" s="12">
+        <v>44261</v>
+      </c>
+      <c r="D129" s="12">
+        <v>44436</v>
+      </c>
+      <c r="E129" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B130" s="1" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C130" s="4"/>
+      <c r="D130" s="4"/>
+      <c r="E130" s="4"/>
+    </row>
+    <row r="131" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B131" s="1" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C131" s="18">
+        <v>45220</v>
+      </c>
+      <c r="D131" s="18">
+        <v>45220</v>
+      </c>
+      <c r="E131" s="14">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="132" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B132" s="1" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C132" s="4"/>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="133" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B133" s="1" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C133" s="15">
+        <v>39760</v>
+      </c>
+      <c r="D133" s="4"/>
+      <c r="E133" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="134" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B134" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C134" s="4"/>
+      <c r="D134" s="4"/>
+      <c r="E134" s="4"/>
+    </row>
+    <row r="135" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B135" s="1" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C135" s="12">
+        <v>45003</v>
+      </c>
+      <c r="D135" s="12">
+        <v>45080</v>
+      </c>
+      <c r="E135" s="14">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="136" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B136" s="1" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C136" s="8">
+        <v>44811</v>
+      </c>
+      <c r="D136" s="8">
+        <v>44811</v>
+      </c>
+      <c r="E136" s="13">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="137" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B137" s="1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C137" s="4"/>
+      <c r="D137" s="4"/>
+      <c r="E137" s="4"/>
+    </row>
+    <row r="138" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B138" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C138" s="12">
+        <v>44739</v>
+      </c>
+      <c r="D138" s="12">
+        <v>44754</v>
+      </c>
+      <c r="E138" s="13">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="139" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B139" s="1" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C139" s="4"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="13">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="140" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B140" s="1" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C140" s="4"/>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4"/>
+    </row>
+    <row r="141" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B141" s="1" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C141" s="4"/>
+      <c r="D141" s="4"/>
+      <c r="E141" s="4"/>
+    </row>
+    <row r="142" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B142" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C142" s="4"/>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4"/>
+    </row>
+    <row r="143" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B143" s="1" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="144" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B144" s="1" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C144" s="4"/>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4"/>
+    </row>
+    <row r="145" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B145" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C145" s="4"/>
+      <c r="D145" s="4"/>
+      <c r="E145" s="4"/>
+    </row>
+    <row r="146" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B146" s="1" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C146" s="4"/>
+      <c r="D146" s="4"/>
+      <c r="E146" s="4"/>
+    </row>
+    <row r="147" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B147" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C147" s="18">
+        <v>45097</v>
+      </c>
+      <c r="D147" s="18">
+        <v>45097</v>
+      </c>
+      <c r="E147" s="14">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="148" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B148" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C148" s="4"/>
+      <c r="D148" s="4"/>
+      <c r="E148" s="4"/>
+    </row>
+    <row r="149" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B149" s="1" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C149" s="4"/>
+      <c r="D149" s="4"/>
+      <c r="E149" s="4"/>
+    </row>
+    <row r="150" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B150" s="1" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C150" s="4"/>
+      <c r="D150" s="4"/>
+      <c r="E150" s="4"/>
+    </row>
+    <row r="151" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B151" s="1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+    </row>
+    <row r="152" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B152" s="1" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C152" s="4"/>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4"/>
+    </row>
+    <row r="153" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B153" s="1" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C153" s="4"/>
+      <c r="D153" s="4"/>
+      <c r="E153" s="4"/>
+    </row>
+    <row r="154" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B154" s="1" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C154" s="11">
+        <v>45423</v>
+      </c>
+      <c r="D154" s="11">
+        <v>45423</v>
+      </c>
+      <c r="E154" s="14">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="155" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B155" s="1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+    </row>
+    <row r="156" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B156" s="1" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C156" s="4"/>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4"/>
+    </row>
+    <row r="157" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B157" s="1" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C157" s="4"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+    </row>
+    <row r="158" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B158" s="1" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C158" s="17">
+        <v>44660</v>
+      </c>
+      <c r="D158" s="17">
+        <v>44674</v>
+      </c>
+      <c r="E158" s="13">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="159" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B159" s="1" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+    </row>
+    <row r="160" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B160" s="1" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C160" s="4"/>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="161" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B161" s="1" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="4"/>
+    </row>
+    <row r="162" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B162" s="1" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C162" s="4"/>
+      <c r="D162" s="4"/>
+      <c r="E162" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="163" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B163" s="1" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="4"/>
+    </row>
+    <row r="164" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B164" s="1" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C164" s="15">
+        <v>42350</v>
+      </c>
+      <c r="D164" s="12">
+        <v>42532</v>
+      </c>
+      <c r="E164" s="13">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="165" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B165" s="1" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="C165" s="4"/>
+      <c r="D165" s="4"/>
+      <c r="E165" s="4"/>
+    </row>
+    <row r="166" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B166" s="3" t="s">
         <v>163</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>